<commit_message>
updated FN & LN in excel
</commit_message>
<xml_diff>
--- a/ScriptingFour/TestData/TestData.xlsx
+++ b/ScriptingFour/TestData/TestData.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\MorningBatch_Combined\Eclipse_Workspace\ScriptingFour\TestData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\MorningBatch_Combined\FinalClone\MorningBatch13JULY2026\ScriptingFour\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48BA8AF9-D3AC-485E-9D81-B6338497F25C}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F596219-0A0D-41B6-9797-7F2B927ED538}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -90,10 +90,10 @@
     <t>TS_102</t>
   </si>
   <si>
-    <t>sg11111</t>
-  </si>
-  <si>
-    <t>user111111</t>
+    <t>sg</t>
+  </si>
+  <si>
+    <t>user1</t>
   </si>
 </sst>
 </file>

</xml_diff>